<commit_message>
DU valuation study: deliverables, verification gates, QC evidence table
16-section Word + 16-sheet formula-first Excel + standalone bibliography,
all rendered to PDF and read as rendered images before delivery. Recalc:
729/729 formula cells reproduce the model, 0 unresolvable, 0 unchecked;
driver test: 22/22 correct-direction, 0 dead inputs. SIGCM and the
model-study depth bar assert clean (gate_check.py). Contested judgement
(post-2026 royalty regime) computed both ways: A 19.14 / B 16.29.
NOT published to the live site per instruction.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3X4qpLFhfa6a9G3h2HreB
</commit_message>
<xml_diff>
--- a/engine/du_study/DU_Valuation_Model_09082026_public.xlsx
+++ b/engine/du_study/DU_Valuation_Model_09082026_public.xlsx
@@ -529,7 +529,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -911,6 +911,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -918,7 +919,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1452,6 +1453,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1459,7 +1461,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1888,6 +1890,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1895,7 +1898,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2387,6 +2390,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2394,7 +2398,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2643,6 +2647,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2650,7 +2655,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3237,6 +3242,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -3244,7 +3250,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4015,6 +4021,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -4022,7 +4029,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4335,6 +4342,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -4342,7 +4350,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4739,6 +4747,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -4746,7 +4755,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -5090,6 +5099,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -5097,7 +5107,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6035,6 +6045,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -6042,7 +6053,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6215,6 +6226,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -6222,7 +6234,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -7172,6 +7184,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -7179,7 +7192,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -7564,6 +7577,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -7571,7 +7585,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -8518,6 +8532,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -8525,7 +8540,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -9197,5 +9212,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
DU study edition 2: beta re-based to FTSE ADX General per instruction
Beta 0.488 (ADX, R2 0.120, n 256, gate passed); DFM General 0.472 and
AE-composite 0.400 published as alternatives. Central 14.98 -> 14.77,
DCF A/B 18.74/15.95, WACC 6.32%->6.08%. All verification gates re-run
green on the rebuilt deliverables (recalc 729/729, driver test 22/22,
scrub/width/figure checks, SIGCM + model-study bar).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3X4qpLFhfa6a9G3h2HreB
</commit_message>
<xml_diff>
--- a/engine/du_study/DU_Valuation_Model_09082026_public.xlsx
+++ b/engine/du_study/DU_Valuation_Model_09082026_public.xlsx
@@ -853,7 +853,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>6.24% -&gt; 6.01% on the AED risk-free path (du has no debt whose cost could define the</t>
+          <t>6.32% -&gt; 6.08% on the AED risk-free path (du has no debt whose cost could define the</t>
         </is>
       </c>
     </row>
@@ -2729,111 +2729,111 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>5.01%</t>
+          <t>5.08%</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>20.09028809929897</v>
+        <v>19.66933438309751</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>22.70200399121432</v>
+        <v>22.15174913365529</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>26.35028687677077</v>
+        <v>25.59094934303363</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>31.80947953617687</v>
+        <v>30.67626651149073</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>40.88093078422291</v>
+        <v>38.96850852166403</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>5.51%</t>
+          <t>5.58%</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>17.70882650142025</v>
+        <v>17.38248029009414</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>19.61381266941501</v>
+        <v>19.20400769626519</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>22.14815500546771</v>
+        <v>21.61270757502213</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>25.68826847930056</v>
+        <v>24.94969675636998</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>30.98549055762803</v>
+        <v>29.88377622565962</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>6.01%</t>
+          <t>6.08%</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>15.85515972490487</v>
+        <v>15.59424768185649</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>17.29553191126147</v>
+        <v>16.9778093008496</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>21.60109684626675</v>
+        <v>21.08026724450918</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>25.03440858808661</v>
+        <v>24.31633715735939</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>6.51%</t>
+          <t>6.58%</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>14.37120518453367</v>
+        <v>14.15746739328381</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>15.49098364095381</v>
+        <v>15.23694854926923</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>16.88724745936135</v>
+        <v>16.57803794656374</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>18.67822143868329</v>
+        <v>18.29028721846222</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>21.06073829814544</v>
+        <v>20.55433959378778</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>7.01%</t>
+          <t>7.08%</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>13.15628173121538</v>
+        <v>12.97770025312425</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>14.04629803516069</v>
+        <v>13.83817789141263</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>15.13119469679048</v>
+        <v>14.88394848792242</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>16.48390668230309</v>
+        <v>16.18310131865233</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>18.218951493052</v>
+        <v>17.84174327636619</v>
       </c>
     </row>
     <row r="12">
@@ -2847,138 +2847,138 @@
       <c r="A13" s="5" t="inlineStr"/>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>5.24%</t>
+          <t>5.32%</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>5.74%</t>
+          <t>5.82%</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>6.24%</t>
+          <t>6.32%</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>6.74%</t>
+          <t>6.82%</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>7.24%</t>
+          <t>7.32%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>terminal 5.01%</t>
+          <t>terminal 5.08%</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>26.99024898628901</v>
+        <v>26.21186590655091</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>26.66777730641833</v>
+        <v>25.89899335245586</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>26.35028687677077</v>
+        <v>25.59094934303363</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>26.03768235944068</v>
+        <v>25.28764153760843</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>25.7298706020608</v>
+        <v>24.98897971072595</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>terminal 5.51%</t>
+          <t>terminal 5.58%</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>22.68454287098371</v>
+        <v>22.13562242012934</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>22.41426634164783</v>
+        <v>21.87213658041468</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>22.14815500546771</v>
+        <v>21.61270757502213</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>21.88612926312696</v>
+        <v>21.35725793786072</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>21.62811133807164</v>
+        <v>21.10571197540687</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>terminal 6.01%</t>
+          <t>terminal 6.08%</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>19.60547307585225</v>
+        <v>19.19660794179827</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>19.37252054004068</v>
+        <v>18.96872899903276</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>18.91729212807279</v>
+        <v>18.52340578337172</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>18.69488112350717</v>
+        <v>18.30582955046258</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>terminal 6.51%</t>
+          <t>terminal 6.58%</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>17.29397218329119</v>
+        <v>16.9769342449448</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>17.08903799568018</v>
+        <v>16.77594593445009</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>16.88724745936135</v>
+        <v>16.57803794656374</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>16.68854067526362</v>
+        <v>16.38315163596903</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>16.49285911301655</v>
+        <v>16.19122969638736</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>terminal 7.01%</t>
+          <t>terminal 7.08%</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>15.49464229835749</v>
+        <v>15.24111786768624</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>15.31151713461568</v>
+        <v>15.06115727875821</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>15.13119469679048</v>
+        <v>14.88394848792242</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>14.95362165989702</v>
+        <v>14.70943918108711</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>14.77874591614142</v>
+        <v>14.53757823737439</v>
       </c>
     </row>
     <row r="20">
@@ -3009,23 +3009,23 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Beta (regression CI ends, then priors)  (0.38 / 0.47 / 0.57 / 0.65 / 0.80)</t>
+          <t>Beta (regression CI ends, then priors)  (0.35 / 0.49 / 0.62 / 0.65 / 0.80)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>19.48137947908612</v>
+        <v>20.32335523048614</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>17.2964558290179</v>
+        <v>16.97182721463749</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>15.43856588369844</v>
+        <v>14.63874519231965</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>14.18617784829437</v>
+        <v>14.19258854611788</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>12.29906647699883</v>
+        <v>12.30464777997424</v>
       </c>
       <c r="H22" s="10">
         <f>MAX(B22:F22)-MIN(B22:F22)</f>
@@ -3039,19 +3039,19 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>20.51089199503732</v>
+        <v>20.08425161688863</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>17.82904430427011</v>
+        <v>17.45699457818922</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>16.67968100822702</v>
+        <v>16.33102727588947</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>15.49200560231583</v>
+        <v>15.16752773017973</v>
       </c>
       <c r="H23" s="10">
         <f>MAX(B23:F23)-MIN(B23:F23)</f>
@@ -3065,19 +3065,19 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>17.14659176130132</v>
+        <v>16.79007037820718</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>18.14487071702368</v>
+        <v>17.76721045267956</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>20.14142862846841</v>
+        <v>19.72149060162431</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>21.13970758419079</v>
+        <v>20.69863067609671</v>
       </c>
       <c r="H24" s="10">
         <f>MAX(B24:F24)-MIN(B24:F24)</f>
@@ -3091,19 +3091,19 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>18.19201125855779</v>
+        <v>17.81339064467879</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>18.66758046565191</v>
+        <v>18.27887058591536</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19.61871887984017</v>
+        <v>19.20983046838851</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>20.0942880869343</v>
+        <v>19.67531040962509</v>
       </c>
       <c r="H25" s="10">
         <f>MAX(B25:F25)-MIN(B25:F25)</f>
@@ -3117,19 +3117,19 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>16.60110760867058</v>
+        <v>16.25397004432989</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>17.87212864070831</v>
+        <v>17.49916028574091</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20.41417070478379</v>
+        <v>19.98954076856297</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>21.68519173682152</v>
+        <v>21.23473100997399</v>
       </c>
       <c r="H26" s="10">
         <f>MAX(B26:F26)-MIN(B26:F26)</f>
@@ -3143,19 +3143,19 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>20.20687199725451</v>
+        <v>19.79009448877729</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>19.67501083500027</v>
+        <v>19.26722250796461</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>18.43400145640707</v>
+        <v>18.04718788606837</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>17.7248532400681</v>
+        <v>17.35002524498481</v>
       </c>
       <c r="H27" s="10">
         <f>MAX(B27:F27)-MIN(B27:F27)</f>
@@ -3169,19 +3169,19 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>19.357486821725</v>
+        <v>18.95677077543478</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>19.26065510581214</v>
+        <v>18.86080506331326</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>19.03471443534881</v>
+        <v>18.63688506836304</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>18.90560548079834</v>
+        <v>18.50893078553434</v>
       </c>
       <c r="H28" s="10">
         <f>MAX(B28:F28)-MIN(B28:F28)</f>
@@ -3195,19 +3195,19 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>18.3125403160204</v>
+        <v>17.93340585281933</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>18.77621646179244</v>
+        <v>18.38610446256195</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>19.3326278367189</v>
+        <v>18.9293427942531</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>19.51264328154805</v>
+        <v>19.10509637215317</v>
       </c>
       <c r="H29" s="10">
         <f>MAX(B29:F29)-MIN(B29:F29)</f>
@@ -3221,19 +3221,19 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>15.85515972490487</v>
+        <v>15.59424768185649</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>17.29553191126147</v>
+        <v>16.9778093008496</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>19.14314967274604</v>
+        <v>18.74435052715193</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>21.60109684626675</v>
+        <v>21.08026724450918</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>25.03440858808661</v>
+        <v>24.31633715735939</v>
       </c>
       <c r="H30" s="10">
         <f>MAX(B30:F30)-MIN(B30:F30)</f>
@@ -4428,14 +4428,14 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>10.96831911684814</v>
+        <v>10.8043265630865</v>
       </c>
       <c r="C5" s="8">
         <f>DCF!C63</f>
         <v/>
       </c>
       <c r="D5" s="7" t="n">
-        <v>29.5836887762623</v>
+        <v>28.73460090831387</v>
       </c>
       <c r="E5" s="9" t="n">
         <v>0.45</v>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>10.96831911684814</v>
+        <v>10.8043265630865</v>
       </c>
     </row>
     <row r="7">
@@ -4840,7 +4840,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>29.5836887762623</v>
+        <v>28.73460090831387</v>
       </c>
     </row>
     <row r="8">
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>16.29100563856143</v>
+        <v>15.94943075692926</v>
       </c>
     </row>
     <row r="20">
@@ -5015,13 +5015,13 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>9.880840632384245</v>
+        <v>9.870305228843574</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>7.824672505907397</v>
+        <v>7.816244183074859</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>11.59431407111495</v>
+        <v>11.58202276698417</v>
       </c>
     </row>
     <row r="25">
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>19.32322520531152</v>
+        <v>18.92260719840512</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>10.18651185142768</v>
+        <v>10.05001098034791</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>22.53703290327117</v>
+        <v>21.99805621498489</v>
       </c>
     </row>
     <row r="26">
@@ -5057,13 +5057,13 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>19.03983619933884</v>
+        <v>18.64224021374001</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>12.64250308760287</v>
+        <v>12.40309632862426</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21.32461654325951</v>
+        <v>20.87930903938881</v>
       </c>
     </row>
     <row r="27">
@@ -5094,7 +5094,7 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>18.08892923382408</v>
+        <v>17.73214262802726</v>
       </c>
     </row>
   </sheetData>
@@ -5776,11 +5776,11 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>Beta (DU weekly vs DFM General Index, 5y)</t>
+          <t>Beta (DU weekly vs FTSE ADX General, 5y)</t>
         </is>
       </c>
       <c r="C52" s="24" t="n">
-        <v>0.472</v>
+        <v>0.488</v>
       </c>
     </row>
     <row r="53">
@@ -8211,7 +8211,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Beta (DU weekly vs its own index, the DFM General, 5 years)</t>
+          <t>Beta (DU weekly vs the FTSE ADX General, 5 years)</t>
         </is>
       </c>
       <c r="C38" s="39">

</xml_diff>

<commit_message>
DU corrected on the growth-basis error
Its terminal was handed a profit figure, a depreciation charge and a working-
capital balance all already grown by (1+g), which the sanctioned construction
grows again. Central 16.8563 -> 16.5778, gap +48.4% -> +45.9%.

The terminal lever reads 16.4935 corrected against the 16.7705 it carried, so
the route is 18.8909 -> 17.1542 -> 16.4935 -> 16.5778 and the cumulative is
-12.24%. It takes more off, not less.

The workbook's own terminal waterfall carried the same growth in its formulas
and is corrected with it, without moving a row -- a dozen formulas on five
other sheets name cells in that block by address.

Study checks: recalc 844 of 844 formula cells with 42 headline
reconciliations, drivers, prose figures and table footing all clean.

One study remains: MODON.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017RcjXG4ETjADcoFJf123yY
</commit_message>
<xml_diff>
--- a/engine/du_study/DU_Valuation_Model_09082026_public.xlsx
+++ b/engine/du_study/DU_Valuation_Model_09082026_public.xlsx
@@ -3183,19 +3183,19 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>18.08333122101619</v>
+        <v>17.78493082128233</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>16.85628211698551</v>
+        <v>16.57779987073647</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>15.6773525856619</v>
+        <v>15.41800738883945</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>14.64621888479577</v>
+        <v>14.40361163207821</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>13.58071406056744</v>
+        <v>13.35540268342493</v>
       </c>
       <c r="H23" s="16">
         <f>MAX(B23:F23)-MIN(B23:F23)</f>
@@ -3209,19 +3209,19 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>14.23093082186519</v>
+        <v>13.99663235400643</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>15.54360646942535</v>
+        <v>15.28721611237145</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>16.85628211698551</v>
+        <v>16.57779987073647</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>18.16895776454566</v>
+        <v>17.86838362910148</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>19.48163341210584</v>
+        <v>19.15896738746652</v>
       </c>
       <c r="H24" s="16">
         <f>MAX(B24:F24)-MIN(B24:F24)</f>
@@ -3235,19 +3235,19 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>16.0030123794334</v>
+        <v>15.7390753752909</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>16.42964724820946</v>
+        <v>16.15843762301369</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>16.85628211698551</v>
+        <v>16.57779987073647</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>17.28291698576156</v>
+        <v>16.99716211845924</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>17.70955185453761</v>
+        <v>17.41652436618203</v>
       </c>
       <c r="H25" s="16">
         <f>MAX(B25:F25)-MIN(B25:F25)</f>
@@ -3261,19 +3261,19 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>17.94035354897293</v>
+        <v>17.64395765095027</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>17.39831783297922</v>
+        <v>17.11087876084336</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>16.85628211698551</v>
+        <v>16.57779987073647</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>16.31424640099178</v>
+        <v>16.04472098062956</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>15.77221068499807</v>
+        <v>15.51164209052265</v>
       </c>
       <c r="H26" s="16">
         <f>MAX(B26:F26)-MIN(B26:F26)</f>
@@ -3287,19 +3287,19 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>13.75255603699058</v>
+        <v>13.52997619908564</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>14.96593768913588</v>
+        <v>14.72151775672866</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>16.85628211698551</v>
+        <v>16.57779987073647</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>17.50551741515849</v>
+        <v>17.21532665438986</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>18.16447323631922</v>
+        <v>17.8623937445068</v>
       </c>
       <c r="H27" s="16">
         <f>MAX(B27:F27)-MIN(B27:F27)</f>
@@ -3313,19 +3313,19 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>17.82633212951094</v>
+        <v>17.53520713489131</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>17.34130712324822</v>
+        <v>17.05650350281389</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>16.85628211698551</v>
+        <v>16.57779987073647</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>16.20958210863521</v>
+        <v>15.9395283612999</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>15.56288210028492</v>
+        <v>15.30125685186333</v>
       </c>
       <c r="H28" s="16">
         <f>MAX(B28:F28)-MIN(B28:F28)</f>
@@ -3339,19 +3339,19 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>17.04752904637536</v>
+        <v>16.76797703305044</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>16.96112886598618</v>
+        <v>16.68206014443815</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>16.85628211698551</v>
+        <v>16.57779987073647</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>16.75952844507809</v>
+        <v>16.48158740434283</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>16.64432820455918</v>
+        <v>16.36703155285978</v>
       </c>
       <c r="H29" s="16">
         <f>MAX(B29:F29)-MIN(B29:F29)</f>
@@ -3365,19 +3365,19 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>17.59954905673535</v>
+        <v>17.30649294892259</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>17.23341326119689</v>
+        <v>16.94753628662998</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>16.85623865313141</v>
+        <v>16.5777572591148</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>16.46769241781963</v>
+        <v>16.19682957743659</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>16.06743170634368</v>
+        <v>15.80441711520527</v>
       </c>
       <c r="H30" s="16">
         <f>MAX(B30:F30)-MIN(B30:F30)</f>
@@ -4594,14 +4594,14 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>10.73766295146378</v>
+        <v>10.56609178209415</v>
       </c>
       <c r="C5" s="8">
         <f>DCF!C63</f>
         <v/>
       </c>
       <c r="D5" s="7" t="n">
-        <v>28.4368006184044</v>
+        <v>27.67129453178129</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -5019,7 +5019,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>10.73766295146378</v>
+        <v>10.56609178209415</v>
       </c>
     </row>
     <row r="7">
@@ -5034,7 +5034,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>28.4368006184044</v>
+        <v>27.67129453178129</v>
       </c>
     </row>
     <row r="8">
@@ -5122,7 +5122,7 @@
         </is>
       </c>
       <c r="C16" s="21" t="n">
-        <v>8.813624287539183</v>
+        <v>8.640808125038413</v>
       </c>
     </row>
     <row r="17">
@@ -8956,11 +8956,11 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Terminal-year operating profit after tax, grown one year (AED mn)</t>
+          <t>FY2030E operating profit after tax — the perpetuity grows this once (AED mn)</t>
         </is>
       </c>
       <c r="C21" s="32">
-        <f>F10*(1+C24)</f>
+        <f>F10</f>
         <v/>
       </c>
     </row>
@@ -9510,11 +9510,11 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>Plus owned depreciation and amortisation, grown one year — the right-of-use charge is neither added back nor charged, which is a lease renewed at its own current cost</t>
+          <t>Plus owned depreciation and amortisation — the right-of-use charge is neither added back nor charged, which is a lease renewed at its own current cost</t>
         </is>
       </c>
       <c r="C74" s="32">
-        <f>2582.418423*(1+C24)</f>
+        <f>2582.418423</f>
         <v/>
       </c>
     </row>
@@ -9536,7 +9536,7 @@
         </is>
       </c>
       <c r="C76" s="32">
-        <f>-C71*10429.868530-C70*-1323.408954</f>
+        <f>-C71*10429.868530-C70*-1297.459758</f>
         <v/>
       </c>
     </row>

</xml_diff>